<commit_message>
feat: Enhance external gateway security and metadata generation
- Added new configuration options in configmap.yaml for HTTP tool settings, including private IP allowance and request size limits.
- Introduced a new Alembic migration (0006_gateway_token_lifecycle.py) to manage token lifecycle and daily quotas for external clients.
- Implemented metadata generation functionality in metadata_generation.py to suggest descriptions for catalog tables and columns using LLM.
- Created comprehensive unit tests for gateway hardening and metadata generation, ensuring robust validation of new features and security measures.
</commit_message>
<xml_diff>
--- a/docs/DataPilot_Spec_Completion_Tracker.xlsx
+++ b/docs/DataPilot_Spec_Completion_Tracker.xlsx
@@ -8,21 +8,22 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Workflows" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enterprise Readiness" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering Health" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Q&amp;A" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bugs Found Live" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priority Order" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sep 2026 Review" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Workflows" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enterprise Readiness" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering Health" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Q&amp;A" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bugs Found Live" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priority Order" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$5:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Core Workflows'!$A$4:$C$58</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Enterprise Readiness'!$A$4:$C$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Engineering Health'!$A$4:$C$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Metadata Q&amp;A'!$A$4:$C$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Bugs Found Live'!$A$4:$F$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Priority Order'!$A$4:$D$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Core Workflows'!$A$4:$C$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Enterprise Readiness'!$A$4:$C$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Engineering Health'!$A$4:$C$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Metadata Q&amp;A'!$A$4:$C$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Bugs Found Live'!$A$4:$F$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Priority Order'!$A$4:$D$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -91,7 +92,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -116,6 +117,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E3F1E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBE9EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF6DE"/>
       </patternFill>
     </fill>
   </fills>
@@ -178,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -208,6 +224,18 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -574,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -602,7 +630,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: docs/IMPLEMENTATION_STATUS_MATRIX.md (11th reconciliation pass, Aug 9 2026) + this session's live click-through verification.</t>
+          <t>Source: docs/IMPLEMENTATION_STATUS_MATRIX.md (eighteenth reconciliation pass, Sep 24 2026 — see §0 and the 'Sep 2026 Review' tab) + live verification on the Docker Compose stack.</t>
         </is>
       </c>
     </row>
@@ -706,7 +734,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Backend suite green (78/79, 1 skipped) and tsc clean as of the last code pass. Demo video and verified screenshots were the two 0% items — now in progress this session.</t>
+          <t>Backend suite green (211 passed, 1 skipped, Sep 24 2026), web tsc clean and 7/7 source tests. Alembic migrations 0001-0006. Demo video still not recorded.</t>
         </is>
       </c>
     </row>
@@ -758,36 +786,60 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>September 2026 review (§0)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>All review findings, Jev decisions, learning loop, analytics picker and the 16 agent/tool/gateway items are done and tested. Open items are user actions (rotate keys, change admin password, commit) and carried-over August items (SSO, pen test, demo video).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="n"/>
-    </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="B15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>Not started / open</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n"/>
+      <c r="B16" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A5:F10"/>
@@ -809,6 +861,1296 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D63"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>September 2026 Review — Closure Tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Devil's-advocate review of UI and API, Jev decision model, learning loop, embedded analytics and agent/tool hardening. Mirrors docs/IMPLEMENTATION_STATUS_MATRIX.md §0 (reconciled Sep 24, 2026; backend 211 passed / 1 skipped, web tsc clean).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Review findings (security, reliability, structure)</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>C1 app DB reachable from user/model SQL</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>STAGING_DATABASE_URL → SELECT-only datapilot_reader; Postgres denies it users (verified live)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Review findings (security, reliability, structure)</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>C2 membership used instead of permission</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>roles.py project role authoritative; viewer blocked from SQL/agents/tools</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Review findings (security, reliability, structure)</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>C3 synchronous ask / lock across LLM calls</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>SSE streaming POST /conversations/{id}/messages/stream; user turn written after generation</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Review findings (security, reliability, structure)</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>C4 blocking calls in async endpoints</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>run_in_threadpool on local agent paths</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Review findings (security, reliability, structure)</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>H1 regex SQL guard</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>sql_guard.py (sqlglot, per dialect) on every execution path</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Review findings (security, reliability, structure)</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>H2 prompt injection</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Untrusted context fenced; catalogued relations only; repair then deterministic fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Review findings (security, reliability, structure)</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>H3 cache</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>SQL only, never rows; TTL; failures never cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Review findings (security, reliability, structure)</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>H4 silent provider fallback</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Per-purpose model_routes; unavailable routed provider → 409</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Review findings (security, reliability, structure)</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>H5 approval not bound to plan</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Frozen plan + plan_hash, verified before every step</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Review findings (security, reliability, structure)</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>H6 Temporal durability</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>One activity per step, idempotency keys, deterministic workflow IDs</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Review findings (security, reliability, structure)</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>M1–M6 (structure, migrations, hot paths, project pinning, auth/secrets, notebook freeze)</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>core.py facade + services/; Alembic 0001–0006; indexes; X-Project-Id; httpOnly cookie + CSRF header; killable notebook cells</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Review findings (security, reliability, structure)</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>Web review items (URLs, 401, cookie auth, a11y, dark mode, TanStack Query, App Router)</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>app/(workspace)/… routes, lib/queries.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Review findings (security, reliability, structure)</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Frictionless (Open Knowledge Foundation) Data Package interchange</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>GET /datapackage, /datasets/{id}/datapackage, validate, descriptive-only import</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Chat, decisions and Jev</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>3-panel Analysis chat rebuilt (threads · answer · inspector)</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>ConversationsView.tsx; route, Jev decision, ensemble, learning sections in the inspector</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Chat, decisions and Jev</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>Data-driven charts (KPI, line, bar, grouped/stacked bar, pie, scatter, table) with a switcher</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>app/charts.py infer_chart; components/charts.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Chat, decisions and Jev</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>Jev as a declared decision-model provider (typesafe/jev-1.13 via OpenRouter)</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>Seeded when OPENROUTER_API_KEY is set; decision models can't serve generation purposes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>Chat, decisions and Jev</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Jev decides route and which agent / query tool</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>Up to 3 agent options (decision_router.local_scores); catalog evidence in Jev's option text</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>Chat, decisions and Jev</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>Jev consequential-action check (escalate only)</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>"Copy all customer records…" escalated at p ≈ 0.9 while rules missed it (live)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>Chat, decisions and Jev</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Jev picks the tool for each agent step</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>_select_step_tools, jev_client.choose_tools; tool_choice evidence in the run trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>Chat, decisions and Jev</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>Jev SQL tie-break</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>sql_candidate_judge on split votes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>Chat, decisions and Jev</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Router's chosen agent carried into the run</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>agent_id on POST /agents/runs; lead agent owns a plan step</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>Chat, decisions and Jev</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Measured accuracy</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>11 labelled routes: Jev 100% (~370 ms), keyword scorer 73%; earlier run Gemini 100% at 1075 ms</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Chat, decisions and Jev</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>Tool-choice evaluation</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>POST /router/evaluate-tools; Learning → Router panel</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>Chat, decisions and Jev</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>Usage per decision type</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>GET /model-usage → by_purpose</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>Chat, decisions and Jev</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>Live proof report</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>scripts/demo_jev_agents.py → docs/demo/; published proof page</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>Chat, decisions and Jev</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>Data residency (keep a project's decisions on-prem)</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>Route decision purposes to the local deterministic model ("on-prem, no external call")</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>Learning loop and SQL</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>Verified-query memory (exact reuse, few-shot, 👍 capture, 👎 review)</t>
+        </is>
+      </c>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>learning.py, routers/learning.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>Learning loop and SQL</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>GEPA prompt optimisation (offline, approval to activate)</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>gepa.py; safety clause always appended</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>Learning loop and SQL</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Multi-model SQL vote with semantic agreement</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>learning.vote_candidates, results_agree</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>Learning loop and SQL</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Cascade vote (the expensive third model only on disagreement)</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>SQL_VOTE_MODE=cascade default; live: 2/2 agreement, Sonnet 5 not called</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>Learning loop and SQL</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>DDL is suggestion-only, driven by slow queries</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>SLOW_QUERY_MS (500); ddl_suggestion artifacts; runs only with ALLOW_DDL_EXECUTION=true + approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>Learning loop and SQL</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>Profiled-only files broke SQL generation</t>
+        </is>
+      </c>
+      <c r="C36" s="15" t="inlineStr">
+        <is>
+          <t>✅ Fixed</t>
+        </is>
+      </c>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>catalog_scope.py; Datasets "profile only" tag</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>Embedded analytics (Superset)</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>"No address associated with hostname"</t>
+        </is>
+      </c>
+      <c r="C37" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>Availability check + guidance; analytics profile documented</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>Embedded analytics (Superset)</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>Blank dashboards (charts taken by other dashboards, text-typed columns, dropped layout rows)</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>Per-dashboard chart names, inferred column types, row wrapping; verified in Superset</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>Embedded analytics (Superset)</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>Dashboard picker: project dashboard, published queries, datasets by source</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>GET /analytics/dashboards, POST /analytics/datasets/{id}/guest-token, SupersetView.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>Embedded analytics (Superset)</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Scope and governance</t>
+        </is>
+      </c>
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
+        <is>
+          <t>Project-scoped; restricted datasets admin-only; PII columns excluded; audited</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>1. Agent configuration read at run time (autonomy cap, provider pin, instructions)</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>2. Budget enforced (reflection counts; AGENT_RUN_MAX_SECONDS; PARTIALLY_SUCCEEDED)</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>3. Built-in tool timeouts; project-scoped sql.preview</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>4. Agent tool calls write ToolExecution rows</t>
+        </is>
+      </c>
+      <c r="C44" s="15" t="inlineStr">
+        <is>
+          <t>✅ (verified live: 7 rows for one run)</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>5. Medium-risk tools only after human approval</t>
+        </is>
+      </c>
+      <c r="C45" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>6. HTTP egress: private-IP block, IP pinning, response cap</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>7. Separation of duties on approvals (APPROVAL_SEPARATION_OF_DUTIES)</t>
+        </is>
+      </c>
+      <c r="C47" s="15" t="inlineStr">
+        <is>
+          <t>✅ (on in Kubernetes)</t>
+        </is>
+      </c>
+      <c r="D47" s="14" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>8. Agent publish gate (AGENT_PUBLISH_MIN_SCORE, audited admin force)</t>
+        </is>
+      </c>
+      <c r="C48" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D48" s="14" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>9. External client token expiry + last used (Alembic 0006)</t>
+        </is>
+      </c>
+      <c r="C49" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D49" s="14" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>10. Rate limiting no longer fails open; list + invoke limited</t>
+        </is>
+      </c>
+      <c r="C50" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D50" s="14" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>11. MCP ping, batch, notifications, JSON-RPC errors</t>
+        </is>
+      </c>
+      <c r="C51" s="15" t="inlineStr">
+        <is>
+          <t>✅ (streamable HTTP GET/SSE not done)</t>
+        </is>
+      </c>
+      <c r="D51" s="14" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>12. Per-grant daily quota</t>
+        </is>
+      </c>
+      <c r="C52" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D52" s="14" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>13. Permission check on /query-tools/{id}/test</t>
+        </is>
+      </c>
+      <c r="C53" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>14. Jev judges split votes</t>
+        </is>
+      </c>
+      <c r="C54" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>15. Tool-choice evaluation</t>
+        </is>
+      </c>
+      <c r="C55" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B56" s="14" t="inlineStr">
+        <is>
+          <t>16. Data residency option</t>
+        </is>
+      </c>
+      <c r="C56" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="14" t="inlineStr">
+        <is>
+          <t>Still open</t>
+        </is>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
+        <is>
+          <t>Rotate the Gemini and OpenRouter API keys shared in chat</t>
+        </is>
+      </c>
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>🔴 User action</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
+        <is>
+          <t>Keys are only in the gitignored .env</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
+        <is>
+          <t>Still open</t>
+        </is>
+      </c>
+      <c r="B58" s="14" t="inlineStr">
+        <is>
+          <t>Change the seeded admin's temporary password</t>
+        </is>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>🔴 User action</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="inlineStr">
+        <is>
+          <t>The forced "change temporary password" dialog still appears</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="14" t="inlineStr">
+        <is>
+          <t>Still open</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
+        <is>
+          <t>Commit this work</t>
+        </is>
+      </c>
+      <c r="C59" s="16" t="inlineStr">
+        <is>
+          <t>🔴 User action</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr">
+        <is>
+          <t>Nothing has been committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>Still open</t>
+        </is>
+      </c>
+      <c r="B60" s="14" t="inlineStr">
+        <is>
+          <t>MCP streamable HTTP (GET/SSE)</t>
+        </is>
+      </c>
+      <c r="C60" s="17" t="inlineStr">
+        <is>
+          <t>🟡 By choice</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="inlineStr">
+        <is>
+          <t>POST JSON-RPC covers current clients</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <t>Still open</t>
+        </is>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
+        <is>
+          <t>AgentVersion.input_schema / config at run time</t>
+        </is>
+      </c>
+      <c r="C61" s="17" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="D61" s="14" t="inlineStr">
+        <is>
+          <t>Stored, not yet used</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>Still open</t>
+        </is>
+      </c>
+      <c r="B62" s="14" t="inlineStr">
+        <is>
+          <t>Timed-out built-in tool threads</t>
+        </is>
+      </c>
+      <c r="C62" s="17" t="inlineStr">
+        <is>
+          <t>🟡 By design</t>
+        </is>
+      </c>
+      <c r="D62" s="14" t="inlineStr">
+        <is>
+          <t>Interrupted at the database; the thread can't be killed</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>Still open</t>
+        </is>
+      </c>
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>Items carried from August (§2): PingFederate SSO, pen test, demo video, connector certification beyond SQL Server</t>
+        </is>
+      </c>
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>🔴 Unchanged</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
+        <is>
+          <t>Outside this review's scope</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1844,7 +3186,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2095,197 +3437,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:C16"/>
-  <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="95" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>3. Engineering / Codebase Health</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Test coverage, architecture, and documentation hygiene.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Detail</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Backend test suite</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>67/68 passing, 1 skipped (test_api.py + test_connection_guard.py), ~9s</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Backend architecture</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>main.py (was 7,069 lines / one file) restructured into a shared module + 25 domain-scoped routers/*.py files; stable across 4+ rounds of concurrent changes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Test coverage breadth</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Single primary test file against 170+ endpoints. Missing dedicated coverage: /lineage/graph, /semantic/graph, /sql/history, /datasets/import, PII masking behavior, RBAC permission-map paths</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Frontend architecture</t>
-        </is>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>page.tsx (was 2,714 lines) restructured into a composition root + types.ts + lib/constants.tsx + 20 component files; tsc --noEmit clean</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Repo cleanliness</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Empty leftover scaffold dirs (apps/web/db, apps/web/worker, apps/web/drizzle, apps/web/app/_sites-preview) remain — permission-locked, needs manual removal from Explorer</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Deployment security posture (OCP/K8s)</t>
-        </is>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Non-root Dockerfiles, securityContext on every Deployment, worker/web HPAs, worker PDB + liveness probe, tunable pool sizing, ingress.example.yaml</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Demo video</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>docs/videos/ was placeholder only as of the last code-level pass. Not recorded yet this session either — deprioritized in favor of the 3 deliverables (this tracker, the consolidated demo doc, the updated PPT) plus the 17 real screenshots below</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Screenshots</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>UPGRADED this session: 32 real screenshots captured by driving the live running app (Chrome, localhost:3000), saved to docs/screenshots/workflows/ — full admin walkthrough (steps 00-13), 3 persona landing pages, plus complete coverage of every remaining nav section (Semantic layer, Tool registry x2, all 6 Admin sub-tabs, Evaluations, live embedded Superset, Analysis, Notebooks, Datasets, Jobs, Artifacts)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:C12"/>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
@@ -2303,7 +3454,7 @@
   <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="95" customWidth="1" min="3" max="3"/>
   </cols>
@@ -2311,21 +3462,21 @@
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>4. Metadata Management — Direct Answers</t>
+          <t>3. Engineering / Codebase Health</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Common product questions, answered directly against the code rather than assumed.</t>
+          <t>Test coverage, architecture, and documentation hygiene.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Question</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -2335,14 +3486,14 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Answer</t>
+          <t>Detail</t>
         </is>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>How does DataPilot pull metadata from a source database?</t>
+          <t>Backend test suite</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -2352,14 +3503,14 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Admin adds a Connector (direct driver or MCP mode), calls POST /connectors/{id}/scan -&gt; discover_metadata(), writes/updates DataAsset rows, raises SchemaDriftEvent on column changes</t>
+          <t>67/68 passing, 1 skipped (test_api.py + test_connection_guard.py), ~9s</t>
         </is>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Can metadata be scanned through an MCP-connected source?</t>
+          <t>Backend architecture</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
@@ -2369,31 +3520,31 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>discover_mcp_metadata() catalogs each upstream tool's schema as a queryable asset with inferred PII/date/id tags</t>
+          <t>main.py (was 7,069 lines / one file) restructured into a shared module + 25 domain-scoped routers/*.py files; stable across 4+ rounds of concurrent changes</t>
         </is>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Can I upload metadata instead of connecting live?</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Test coverage breadth</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>POST /datasets/import accepts a CSV, creates/updates DataAsset rows tagged metadata_status="manual_import", no live connection required</t>
+          <t>Single primary test file against 170+ endpoints. Missing dedicated coverage: /lineage/graph, /semantic/graph, /sql/history, /datasets/import, PII masking behavior, RBAC permission-map paths</t>
         </is>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Can I manually edit or review scanned metadata (description, tags, owner, sensitivity, freshness, status)?</t>
+          <t>Frontend architecture</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -2403,31 +3554,31 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>PUT /datasets/{asset_id} — API and the DatasetsView.tsx edit modal both cover all six fields</t>
+          <t>page.tsx (was 2,714 lines) restructured into a composition root + types.ts + lib/constants.tsx + 20 component files; tsc --noEmit clean</t>
         </is>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Is discovered/ingested metadata flagged for PII?</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Repo cleanliness</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>annotate_columns() in app/pii.py tags columns with sensitivity: "pii" + pii_category during file ingestion and connector metadata discovery</t>
+          <t>Empty leftover scaffold dirs (apps/web/db, apps/web/worker, apps/web/drizzle, apps/web/app/_sites-preview) remain — permission-locked, needs manual removal from Explorer</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Is metadata scoped per project?</t>
+          <t>Deployment security posture (OCP/K8s)</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
@@ -2437,14 +3588,14 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>DataAsset.project_id / Connector.project_id are FKs, every route filters by require_current_project(). No cross-project catalog sharing</t>
+          <t>Non-root Dockerfiles, securityContext on every Deployment, worker/web HPAs, worker PDB + liveness probe, tunable pool sizing, ingress.example.yaml</t>
         </is>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Can one project have multiple sets of joined tables, or multiple "data models"/groupings?</t>
+          <t>Demo video</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
@@ -2454,14 +3605,14 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Confirmed no such concept exists in code — a project's catalog is a flat list of DataAsset rows. Only grouping primitives are free-text tags and schema_name. No first-class "data model"/"domain" object. This is a design decision (new entity + migration + UI), not a bug</t>
+          <t>docs/videos/ was placeholder only as of the last code-level pass. Not recorded yet this session either — deprioritized in favor of the 3 deliverables (this tracker, the consolidated demo doc, the updated PPT) plus the 17 real screenshots below</t>
         </is>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Where are business names for tables/columns stored, and do they reach the vector store?</t>
+          <t>Screenshots</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
@@ -2471,7 +3622,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Postgres (DataAsset.description, DataAsset.columns JSON) is the source of truth; reaches Qdrant via index_document(). embed_text() now calls the active ModelProvider's real embeddings API (Gemini / OpenAI / OpenAI-compatible) using ModelProvider.embedding_model — falls back to a deterministic hash only when no provider/secret is configured or the provider type has no embeddings API</t>
+          <t>UPGRADED this session: 32 real screenshots captured by driving the live running app (Chrome, localhost:3000), saved to docs/screenshots/workflows/ — full admin walkthrough (steps 00-13), 3 persona landing pages, plus complete coverage of every remaining nav section (Semantic layer, Tool registry x2, all 6 Admin sub-tabs, Evaluations, live embedded Superset, Analysis, Notebooks, Datasets, Jobs, Artifacts)</t>
         </is>
       </c>
     </row>
@@ -2486,6 +3637,197 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>4. Metadata Management — Direct Answers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Common product questions, answered directly against the code rather than assumed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>How does DataPilot pull metadata from a source database?</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Admin adds a Connector (direct driver or MCP mode), calls POST /connectors/{id}/scan -&gt; discover_metadata(), writes/updates DataAsset rows, raises SchemaDriftEvent on column changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Can metadata be scanned through an MCP-connected source?</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>discover_mcp_metadata() catalogs each upstream tool's schema as a queryable asset with inferred PII/date/id tags</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Can I upload metadata instead of connecting live?</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>POST /datasets/import accepts a CSV, creates/updates DataAsset rows tagged metadata_status="manual_import", no live connection required</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Can I manually edit or review scanned metadata (description, tags, owner, sensitivity, freshness, status)?</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>PUT /datasets/{asset_id} — API and the DatasetsView.tsx edit modal both cover all six fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Is discovered/ingested metadata flagged for PII?</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>annotate_columns() in app/pii.py tags columns with sensitivity: "pii" + pii_category during file ingestion and connector metadata discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Is metadata scoped per project?</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>DataAsset.project_id / Connector.project_id are FKs, every route filters by require_current_project(). No cross-project catalog sharing</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Can one project have multiple sets of joined tables, or multiple "data models"/groupings?</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Confirmed no such concept exists in code — a project's catalog is a flat list of DataAsset rows. Only grouping primitives are free-text tags and schema_name. No first-class "data model"/"domain" object. This is a design decision (new entity + migration + UI), not a bug</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Where are business names for tables/columns stored, and do they reach the vector store?</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Postgres (DataAsset.description, DataAsset.columns JSON) is the source of truth; reaches Qdrant via index_document(). embed_text() now calls the active ModelProvider's real embeddings API (Gemini / OpenAI / OpenAI-compatible) using ModelProvider.embedding_model — falls back to a deterministic hash only when no provider/secret is configured or the provider type has no embeddings API</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:C12"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2654,13 +3996,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2713,7 +4055,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Good demo</t>
+          <t>Security hygiene (user action)</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
@@ -2723,7 +4065,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Record the actual demo video. Screenshots DONE this session — 32 captured, full application coverage (up from 17). Run one live SQL Server scan end-to-end (direct + MCP) against the now-unblocked sqlserver-demo container</t>
+          <t>Rotate the Gemini and OpenRouter API keys shared in chat; change the seeded admin's temporary password; commit the September review work (nothing is committed yet).</t>
         </is>
       </c>
     </row>
@@ -2735,7 +4077,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Enterprise credibility</t>
+          <t>Good demo</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
@@ -2745,29 +4087,29 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>SSO completion, live connector certification beyond SQL Server (Oracle/Teradata/BigQuery), a real security review/pen test, a NetworkPolicy, a backup/restore drill</t>
+          <t>Record the actual demo video. Screenshots DONE this session — 32 captured, full application coverage (up from 17). Run one live SQL Server scan end-to-end (direct + MCP) against the now-unblocked sqlserver-demo container</t>
         </is>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Correctness / trust</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Enterprise credibility</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>artifacts.py's approval-decision endpoint is the one remaining raw user.role check (real migration gap). Re-verify require_permission/project_permissions/current_membership imports stay intact after future refactors. Give tests/test_new_endpoints.py its own isolated DATABASE_URL. Add automated PII-masking tests</t>
+          <t>SSO completion, live connector certification beyond SQL Server (Oracle/Teradata/BigQuery), a real security review/pen test, a NetworkPolicy, a backup/restore drill</t>
         </is>
       </c>
     </row>
@@ -2779,17 +4121,17 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Scale-readiness</t>
-        </is>
-      </c>
-      <c r="C8" s="13" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Correctness / trust</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Load-test against the documented Postgres connection-pool math before raising HPA maxReplicas. Add a NetworkPolicy. Consider a custom Temporal-queue-depth autoscaling metric for the worker</t>
+          <t>artifacts.py's approval-decision endpoint is the one remaining raw user.role check (real migration gap). Re-verify require_permission/project_permissions/current_membership imports stay intact after future refactors. Give tests/test_new_endpoints.py its own isolated DATABASE_URL. Add automated PII-masking tests</t>
         </is>
       </c>
     </row>
@@ -2801,7 +4143,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Usability</t>
+          <t>Scale-readiness</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -2811,7 +4153,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Add filter controls to the query-tool gateway list — the one remaining piece of "registry marketplace" polish</t>
+          <t>Load-test against the documented Postgres connection-pool math before raising HPA maxReplicas. Add a NetworkPolicy. Consider a custom Temporal-queue-depth autoscaling metric for the worker</t>
         </is>
       </c>
     </row>
@@ -2823,37 +4165,59 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Maintainability</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Usability</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>main.py and page.tsx split into per-domain/per-view modules, verified stable across 4+ rounds of unrelated concurrent changes</t>
+          <t>Add filter controls to the query-tool gateway list — the one remaining piece of "registry marketplace" polish</t>
         </is>
       </c>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Maintainability</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>main.py and page.tsx split into per-domain/per-view modules, verified stable across 4+ rounds of unrelated concurrent changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Embedding model wiring</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>ModelProvider.embedding_model now actually wired into vector_store.embed_text() for Gemini/OpenAI/OpenAI-compatible, with dimension-safe reindexing. Remaining open item: a first-class grouping entity if multi-model-per-project becomes a real requirement</t>
         </is>

</xml_diff>

<commit_message>
feat: Implement AI-suggested metadata, paste-SQL explain mode, and export functionality
- Added AI-suggested metadata generation for tables and columns during import, with human-editable options.
- Introduced a new endpoint for pasting SQL queries to receive explanations in business terms.
- Enabled export options for catalog data in CSV format and semantic graph data in JSON/SVG formats.
- Enhanced semantic relationship graph readability with a physics simulation for node layout, ensuring clear visual representation.
- Fixed multiple bugs related to metadata overwriting and graph rendering.
- Verified all features with new tests and live browser checks against the Docker Compose stack.
</commit_message>
<xml_diff>
--- a/docs/DataPilot_Spec_Completion_Tracker.xlsx
+++ b/docs/DataPilot_Spec_Completion_Tracker.xlsx
@@ -630,7 +630,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: docs/IMPLEMENTATION_STATUS_MATRIX.md (eighteenth reconciliation pass, Sep 24 2026 — see §0 and the 'Sep 2026 Review' tab) + live verification on the Docker Compose stack.</t>
+          <t>Source: docs/IMPLEMENTATION_STATUS_MATRIX.md (nineteenth reconciliation pass, Sep 24 2026 — §0 September review on the 'Sep 2026 Review' tab; §1 additions for AI-suggested metadata, paste-SQL explain and catalog/graph export) + live verification on the Docker Compose stack.</t>
         </is>
       </c>
     </row>
@@ -673,10 +673,10 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>1</v>
@@ -810,6 +810,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
@@ -2151,7 +2152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2521,12 +2522,12 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>✅ Real cross-source bug fixed, then corrected further for MCP connectors — see seventeenth-pass change-log entry</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>GET /semantic/graph — governed joins + inferred column-matched suggestions flagged for review</t>
+          <t>GET /semantic/graph — nodes from DataAsset, edges from governed SemanticJoinPolicy plus inferred column-name-matched suggestions flagged governed: false for review. Was suggesting joins across completely different external connectors (e.g. a Postgres warehouse and a SQL Server warehouse that both happen to have a customer_id column) purely because column names matched, with no notion that /sql/generate//sql/execute are always scoped to one connector (or the local workspace) at a time — those joins can never actually execute. User caught this live, from the graph rendering as a dense, near-fully-connected mesh with no visible structure. Fixed (fifteenth pass): inferred edges confined to assets that share a group_key(), each node carries a new group/source_label field, and the frontend clusters nodes into per-source arcs with distinct colors and a legend instead of one flat ring; POST/PUT /semantic/joins (validate_semantic_join_policy()) rejects a governed policy across two different connectors (422). User caught a second, deeper issue (seventeenth pass): that connector-level grouping is only correct for direct-driver connectors. An MCP-backed connector's assets are individually-discovered *tools* (discover_mcp_metadata() hardcodes schema_name="mcp" regardless of what backend a tool actually fronts), MCP execution invokes exactly one named tool per call with zero cross-tool join path anywhere in the runtime, and a single MCP toolbox can front more than one physically distinct backend (confirmed via infra/mcp-toolbox/toolbox.yaml's two separate kind: source blocks) — so two tools on the very same connector must never be treated as joinable either. group_key() and validate_semantic_join_policy() now branch on connection_mode: direct connectors keep one bucket per connector_id; MCP connectors key every asset individually. The graph UI still colors/legends by source_label (so an MCP toolbox reads as one color, not N), while arc placement uses the finer-grained group so its tools render as visually distinct, non-linked clusters. Retrieval/generation itself was independently verified NOT to have the original cross-connector problem — see the grouping row in §4 below. Nineteenth-pass addendum: the grouping/coloring above was correct but the label rendering wasn't — a fixed 900×460 canvas and a hardcoded 14px label offset meant a real ~33-node catalog (this session's live test) produced overlapping text once more than a handful of nodes shared a tight angular range, independent of the grouping fix. SemanticGraphPanel now scales canvas radius with node count, staggers label offsets for nodes placed close together on the ring (deterministic, no DOM measurement), and adds a node filter box and manual zoom for dense graphs. Verified live against the 24-inferred-edge/33-node catalog: labels no longer overlap and the filter correctly dims non-matching nodes without reflowing the layout</t>
         </is>
       </c>
     </row>
@@ -3173,6 +3174,57 @@
       <c r="C62" s="4" t="inlineStr">
         <is>
           <t>Ran "Profile demo.customers: row count, null rates, and the distribution of customer_id" from the Workspace ask box. Plan/trace shows Planner -&gt; Metadata -&gt; SQL Analyst -&gt; Quality -&gt; Policy, all COMPLETE; run correctly paused at "WAITING FOR APPROVAL" (deterministic policy gate, HIGH risk), was approved via the Approvals inbox, and the job reached SUCCEEDED with 11 evidence items and a full execution log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>Catalog + semantic-graph export</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>✅ New this session</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>The backend Data Package export (GET /datapackage, GET /datasets/{id}/datapackage, frictionless.py) existed with no frontend button — DatasetsView.tsx now has "Export CSV" (client-side, one row per column: schema/table/column/type/business_name/description/tags/owner/sensitivity/status) and "Export data package" (downloads the existing JSON endpoint's response). SemanticGraphPanel (SemanticView.tsx) gained "Export graph data (JSON)" and "Export as SVG" (a visual snapshot only — the exported file doesn't carry globals.css's node/edge styling, so it renders unstyled outside the app; noted inline in the code)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>LLM-suggested table/column descriptions</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>✅ New this session</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>app/metadata_generation.py's suggest_dataset_metadata() asks the project's routed model (new purpose metadata_generation) for a table description plus per-column business_name/description, from column names/types only — never sample row values, since a description doesn't need them and they could carry PII into a third-party call. Auto-applied (status ai_suggested) the first time a table is discovered via connector scan (metadata_scan_runtime.py) or file ingest/staging (routers/files.py, both the direct-ingest and mapped-staging paths), gated by is_unreviewed_description() so a rescan can never clobber a human-written or already-suggested description — a real overwrite bug in this exact gate was found and fixed mid-session (see change log). Also exposed as an on-demand POST /datasets/{asset_id}/generate-metadata ("Generate with AI" in the Review-metadata modal) that returns a suggestion for the human to edit/save through the existing flow rather than writing to the DB itself; saving an ai_suggested dataset without picking a different status auto-promotes it to reviewed. 9 new unit tests (test_metadata_generation.py) cover empty/malformed/erroring provider responses, an invented column name being dropped, and description truncation</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>Paste-your-own-SQL explain/validate mode</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>✅ New this session</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>POST /sql/explain (routers/sql.py) lets a user paste a hand-written statement instead of asking in natural language: runs the exact same read-only/catalog-only guard as generation (_safe_read_only_sql + unknown_relations, scoped through catalog_scope.queryable_asset_ids like /sql/generate), then asks the model to explain it in business terms and returns a response shaped exactly like /sql/generate's so the SQL workspace's existing evidence/preview panels render it with no new UI logic. SQLView.tsx gets an "Ask a question" / "Paste SQL" mode toggle plus a "Save as verified query" action that registers the explained SQL through the existing POST /verified-queries. The NL path also gained an optional "Add extra context" field folded into the question text sent to /sql/generate — no backend schema change needed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add interactive charts and graph canvas styles
- Introduced `charts-interactive.css` for enhanced chart interactions including toolbars, breadcrumbs, and tooltips.
- Added `graph-canvas.css` for styling the interactive graph canvas, including node and edge styles, toolbars, and responsive design.
- Implemented media queries for reduced motion and mobile responsiveness.

docs: Consolidate UX documentation for improved navigation

- Created `UX_CONSOLIDATION.md` to outline the strategy for merging, hiding, or removing redundant screens and features.
- Detailed inventory of existing sidebar items and identified overlaps for better organization by user roles.

feat: Initialize Retail Banking database with sample data

- Added `retail_banking.sql` to create the RetailBanking database with schemas, tables, and deterministic sample data for testing.
- Ensured idempotency to allow safe execution on every container start.
</commit_message>
<xml_diff>
--- a/docs/DataPilot_Spec_Completion_Tracker.xlsx
+++ b/docs/DataPilot_Spec_Completion_Tracker.xlsx
@@ -630,7 +630,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: docs/IMPLEMENTATION_STATUS_MATRIX.md (nineteenth reconciliation pass, Sep 24 2026 — §0 September review on the 'Sep 2026 Review' tab; §1 additions for AI-suggested metadata, paste-SQL explain and catalog/graph export) + live verification on the Docker Compose stack.</t>
+          <t>Source: docs/IMPLEMENTATION_STATUS_MATRIX.md (eighteenth reconciliation pass, Sep 24 2026 — see §0 and the 'Sep 2026 Review' tab) + live verification on the Docker Compose stack.</t>
         </is>
       </c>
     </row>
@@ -793,10 +793,10 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>3</v>
@@ -810,7 +810,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
@@ -862,7 +861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1614,136 +1613,144 @@
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>Embedded analytics (Superset)</t>
+          <t>Learning loop and SQL</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>"No address associated with hostname"</t>
+          <t>Column / schema questions ran unrelated SQL</t>
         </is>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>✅ Fixed</t>
         </is>
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
-          <t>Availability check + guidance; analytics profile documented</t>
+          <t>catalog_answer.py: answered from catalog metadata, no SQL; "this / closest table" follows the conversation across sources</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>Embedded analytics (Superset)</t>
+          <t>Learning loop and SQL</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>Blank dashboards (charts taken by other dashboards, text-typed columns, dropped layout rows)</t>
+          <t>Rejected model SQL silently replaced by a generic fallback shown as PASSED</t>
         </is>
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>✅ Fixed</t>
         </is>
       </c>
       <c r="D38" s="14" t="inlineStr">
         <is>
-          <t>Per-dashboard chart names, inferred column types, row wrapping; verified in Superset</t>
+          <t>Status "fallback" + the answer says the result may not answer the question</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>Embedded analytics (Superset)</t>
+          <t>Learning loop and SQL</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>Dashboard picker: project dashboard, published queries, datasets by source</t>
+          <t>Follow-up after reload ran on the wrong source</t>
         </is>
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>✅ Fixed</t>
         </is>
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
-          <t>GET /analytics/dashboards, POST /analytics/datasets/{id}/guest-token, SupersetView.tsx</t>
+          <t>Source picker restores the conversation's last source</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>Embedded analytics (Superset)</t>
+          <t>Learning loop and SQL</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>Scope and governance</t>
+          <t>"Banking demo warehouse" was catalog-only (no credentials)</t>
         </is>
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>✅ Fixed</t>
         </is>
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
-          <t>Project-scoped; restricted datasets admin-only; PII columns excluded; audited</t>
+          <t>Live RetailBanking DB in sqlserver-demo (infra/sqlserver-init/retail_banking.sql); connector wired to env:SQLSERVER_DEMO_CREDENTIALS</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>Agents, tools and external gateway (16 items)</t>
+          <t>Learning loop and SQL</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>1. Agent configuration read at run time (autonomy cap, provider pin, instructions)</t>
+          <t>Query-tool suggestions from another source</t>
         </is>
       </c>
       <c r="C41" s="15" t="inlineStr">
         <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D41" s="14" t="inlineStr"/>
+          <t>✅ Fixed</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>decide(..., connector_id) only offers tools for the selected source</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>Agents, tools and external gateway (16 items)</t>
+          <t>Learning loop and SQL</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>2. Budget enforced (reflection counts; AGENT_RUN_MAX_SECONDS; PARTIALLY_SUCCEEDED)</t>
+          <t>SQL Server decimals stored as text (charts fell back to tables)</t>
         </is>
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D42" s="14" t="inlineStr"/>
+          <t>✅ Fixed</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>charts.json_default keeps DECIMAL numeric</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>Agents, tools and external gateway (16 items)</t>
+          <t>Learning loop and SQL</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>3. Built-in tool timeouts; project-scoped sql.preview</t>
+          <t>One-click "Publish to Superset" from a chat answer; resizable chat panels</t>
         </is>
       </c>
       <c r="C43" s="15" t="inlineStr">
@@ -1751,35 +1758,43 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D43" s="14" t="inlineStr"/>
+      <c r="D43" s="14" t="inlineStr">
+        <is>
+          <t>POST /analytics/publish-message; draggable History / Inspector widths</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>Agents, tools and external gateway (16 items)</t>
+          <t>Embedded analytics (Superset)</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>4. Agent tool calls write ToolExecution rows</t>
+          <t>"No address associated with hostname"</t>
         </is>
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>✅ (verified live: 7 rows for one run)</t>
-        </is>
-      </c>
-      <c r="D44" s="14" t="inlineStr"/>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>Availability check + guidance; analytics profile documented</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>Agents, tools and external gateway (16 items)</t>
+          <t>Embedded analytics (Superset)</t>
         </is>
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>5. Medium-risk tools only after human approval</t>
+          <t>Blank dashboards (charts taken by other dashboards, text-typed columns, dropped layout rows)</t>
         </is>
       </c>
       <c r="C45" s="15" t="inlineStr">
@@ -1787,17 +1802,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D45" s="14" t="inlineStr"/>
+      <c r="D45" s="14" t="inlineStr">
+        <is>
+          <t>Per-dashboard chart names, inferred column types, row wrapping; verified in Superset</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t>Agents, tools and external gateway (16 items)</t>
+          <t>Embedded analytics (Superset)</t>
         </is>
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>6. HTTP egress: private-IP block, IP pinning, response cap</t>
+          <t>Dashboard picker: project dashboard, published queries, datasets by source</t>
         </is>
       </c>
       <c r="C46" s="15" t="inlineStr">
@@ -1805,25 +1824,33 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D46" s="14" t="inlineStr"/>
+      <c r="D46" s="14" t="inlineStr">
+        <is>
+          <t>GET /analytics/dashboards, POST /analytics/datasets/{id}/guest-token, SupersetView.tsx</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>Agents, tools and external gateway (16 items)</t>
+          <t>Embedded analytics (Superset)</t>
         </is>
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>7. Separation of duties on approvals (APPROVAL_SEPARATION_OF_DUTIES)</t>
+          <t>Scope and governance</t>
         </is>
       </c>
       <c r="C47" s="15" t="inlineStr">
         <is>
-          <t>✅ (on in Kubernetes)</t>
-        </is>
-      </c>
-      <c r="D47" s="14" t="inlineStr"/>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D47" s="14" t="inlineStr">
+        <is>
+          <t>Project-scoped; restricted datasets admin-only; PII columns excluded; audited</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="14" t="inlineStr">
@@ -1833,7 +1860,7 @@
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>8. Agent publish gate (AGENT_PUBLISH_MIN_SCORE, audited admin force)</t>
+          <t>1. Agent configuration read at run time (autonomy cap, provider pin, instructions)</t>
         </is>
       </c>
       <c r="C48" s="15" t="inlineStr">
@@ -1851,7 +1878,7 @@
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>9. External client token expiry + last used (Alembic 0006)</t>
+          <t>2. Budget enforced (reflection counts; AGENT_RUN_MAX_SECONDS; PARTIALLY_SUCCEEDED)</t>
         </is>
       </c>
       <c r="C49" s="15" t="inlineStr">
@@ -1869,7 +1896,7 @@
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>10. Rate limiting no longer fails open; list + invoke limited</t>
+          <t>3. Built-in tool timeouts; project-scoped sql.preview</t>
         </is>
       </c>
       <c r="C50" s="15" t="inlineStr">
@@ -1887,12 +1914,12 @@
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>11. MCP ping, batch, notifications, JSON-RPC errors</t>
+          <t>4. Agent tool calls write ToolExecution rows</t>
         </is>
       </c>
       <c r="C51" s="15" t="inlineStr">
         <is>
-          <t>✅ (streamable HTTP GET/SSE not done)</t>
+          <t>✅ (verified live: 7 rows for one run)</t>
         </is>
       </c>
       <c r="D51" s="14" t="inlineStr"/>
@@ -1905,7 +1932,7 @@
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>12. Per-grant daily quota</t>
+          <t>5. Medium-risk tools only after human approval</t>
         </is>
       </c>
       <c r="C52" s="15" t="inlineStr">
@@ -1923,7 +1950,7 @@
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>13. Permission check on /query-tools/{id}/test</t>
+          <t>6. HTTP egress: private-IP block, IP pinning, response cap</t>
         </is>
       </c>
       <c r="C53" s="15" t="inlineStr">
@@ -1941,12 +1968,12 @@
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>14. Jev judges split votes</t>
+          <t>7. Separation of duties on approvals (APPROVAL_SEPARATION_OF_DUTIES)</t>
         </is>
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>✅ (on in Kubernetes)</t>
         </is>
       </c>
       <c r="D54" s="14" t="inlineStr"/>
@@ -1959,7 +1986,7 @@
       </c>
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>15. Tool-choice evaluation</t>
+          <t>8. Agent publish gate (AGENT_PUBLISH_MIN_SCORE, audited admin force)</t>
         </is>
       </c>
       <c r="C55" s="15" t="inlineStr">
@@ -1977,7 +2004,7 @@
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>16. Data residency option</t>
+          <t>9. External client token expiry + last used (Alembic 0006)</t>
         </is>
       </c>
       <c r="C56" s="15" t="inlineStr">
@@ -1990,152 +2017,498 @@
     <row r="57">
       <c r="A57" s="14" t="inlineStr">
         <is>
-          <t>Still open</t>
+          <t>Agents, tools and external gateway (16 items)</t>
         </is>
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>Rotate the Gemini and OpenRouter API keys shared in chat</t>
-        </is>
-      </c>
-      <c r="C57" s="16" t="inlineStr">
-        <is>
-          <t>🔴 User action</t>
-        </is>
-      </c>
-      <c r="D57" s="14" t="inlineStr">
-        <is>
-          <t>Keys are only in the gitignored .env</t>
-        </is>
-      </c>
+          <t>10. Rate limiting no longer fails open; list + invoke limited</t>
+        </is>
+      </c>
+      <c r="C57" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="14" t="inlineStr">
         <is>
-          <t>Still open</t>
+          <t>Agents, tools and external gateway (16 items)</t>
         </is>
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>Change the seeded admin's temporary password</t>
-        </is>
-      </c>
-      <c r="C58" s="16" t="inlineStr">
-        <is>
-          <t>🔴 User action</t>
-        </is>
-      </c>
-      <c r="D58" s="14" t="inlineStr">
-        <is>
-          <t>The forced "change temporary password" dialog still appears</t>
-        </is>
-      </c>
+          <t>11. MCP ping, batch, notifications, JSON-RPC errors</t>
+        </is>
+      </c>
+      <c r="C58" s="15" t="inlineStr">
+        <is>
+          <t>✅ (streamable HTTP GET/SSE not done)</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="14" t="inlineStr">
         <is>
-          <t>Still open</t>
+          <t>Agents, tools and external gateway (16 items)</t>
         </is>
       </c>
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t>Commit this work</t>
-        </is>
-      </c>
-      <c r="C59" s="16" t="inlineStr">
-        <is>
-          <t>🔴 User action</t>
-        </is>
-      </c>
-      <c r="D59" s="14" t="inlineStr">
-        <is>
-          <t>Nothing has been committed</t>
-        </is>
-      </c>
+          <t>12. Per-grant daily quota</t>
+        </is>
+      </c>
+      <c r="C59" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="14" t="inlineStr">
         <is>
-          <t>Still open</t>
+          <t>Agents, tools and external gateway (16 items)</t>
         </is>
       </c>
       <c r="B60" s="14" t="inlineStr">
         <is>
-          <t>MCP streamable HTTP (GET/SSE)</t>
-        </is>
-      </c>
-      <c r="C60" s="17" t="inlineStr">
-        <is>
-          <t>🟡 By choice</t>
-        </is>
-      </c>
-      <c r="D60" s="14" t="inlineStr">
-        <is>
-          <t>POST JSON-RPC covers current clients</t>
-        </is>
-      </c>
+          <t>13. Permission check on /query-tools/{id}/test</t>
+        </is>
+      </c>
+      <c r="C60" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="14" t="inlineStr">
         <is>
-          <t>Still open</t>
+          <t>Agents, tools and external gateway (16 items)</t>
         </is>
       </c>
       <c r="B61" s="14" t="inlineStr">
         <is>
-          <t>AgentVersion.input_schema / config at run time</t>
-        </is>
-      </c>
-      <c r="C61" s="17" t="inlineStr">
-        <is>
-          <t>🟡</t>
-        </is>
-      </c>
-      <c r="D61" s="14" t="inlineStr">
-        <is>
-          <t>Stored, not yet used</t>
-        </is>
-      </c>
+          <t>14. Jev judges split votes</t>
+        </is>
+      </c>
+      <c r="C61" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D61" s="14" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="14" t="inlineStr">
         <is>
-          <t>Still open</t>
+          <t>Agents, tools and external gateway (16 items)</t>
         </is>
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>Timed-out built-in tool threads</t>
-        </is>
-      </c>
-      <c r="C62" s="17" t="inlineStr">
-        <is>
-          <t>🟡 By design</t>
-        </is>
-      </c>
-      <c r="D62" s="14" t="inlineStr">
-        <is>
-          <t>Interrupted at the database; the thread can't be killed</t>
-        </is>
-      </c>
+          <t>15. Tool-choice evaluation</t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D62" s="14" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="14" t="inlineStr">
         <is>
+          <t>Agents, tools and external gateway (16 items)</t>
+        </is>
+      </c>
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>16. Data residency option</t>
+        </is>
+      </c>
+      <c r="C63" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <t>Learning, building, agents, graphs and consolidation (Sep 24–25)</t>
+        </is>
+      </c>
+      <c r="B64" s="14" t="inlineStr">
+        <is>
+          <t>Plan-guided query tuner: equivalence-checked rewrites (up to 6–8 attempts), no index creation, apply only via approval</t>
+        </is>
+      </c>
+      <c r="C64" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D64" s="14" t="inlineStr">
+        <is>
+          <t>query_tuner.py, POST /sql/tune, Learning → Performance; live: 2.71 → 1.98 ms (27%) with 3 equivalent attempts</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="14" t="inlineStr">
+        <is>
+          <t>Learning, building, agents, graphs and consolidation (Sep 24–25)</t>
+        </is>
+      </c>
+      <c r="B65" s="14" t="inlineStr">
+        <is>
+          <t>Paste &amp; run any-length SQL, plan analysis in plain language, full / piece-wise (per-CTE) rewrite</t>
+        </is>
+      </c>
+      <c r="C65" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D65" s="14" t="inlineStr">
+        <is>
+          <t>POST /sql/run, POST /sql/analyze; 1,000+ line query ran live; piece-wise rewrite accepted only if the whole result matches</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="14" t="inlineStr">
+        <is>
+          <t>Learning, building, agents, graphs and consolidation (Sep 24–25)</t>
+        </is>
+      </c>
+      <c r="B66" s="14" t="inlineStr">
+        <is>
+          <t>Build very large SQL from business logic (plan → per-step build + repair → one WITH query)</t>
+        </is>
+      </c>
+      <c r="C66" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D66" s="14" t="inlineStr">
+        <is>
+          <t>sql_composer.py, /sql/compose/*, SQL → Build from business logic; 65-step plan in tests, 7-step plan live</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="14" t="inlineStr">
+        <is>
+          <t>Learning, building, agents, graphs and consolidation (Sep 24–25)</t>
+        </is>
+      </c>
+      <c r="B67" s="14" t="inlineStr">
+        <is>
+          <t>Reviewer agent: every chat answer gets ok / check / doubtful with checks + Jev probabilities</t>
+        </is>
+      </c>
+      <c r="C67" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D67" s="14" t="inlineStr">
+        <is>
+          <t>answer_review.py; live verdict ok 0.90 via Jev</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>Learning, building, agents, graphs and consolidation (Sep 24–25)</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>Draft with AI for new agents and query tools (registry-only tools)</t>
+        </is>
+      </c>
+      <c r="C68" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D68" s="14" t="inlineStr">
+        <is>
+          <t>agent_designer.py, POST /agents/draft, POST /query-tools/draft; Jev + design model picks, validated</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>Learning, building, agents, graphs and consolidation (Sep 24–25)</t>
+        </is>
+      </c>
+      <c r="B69" s="14" t="inlineStr">
+        <is>
+          <t>Interactive charts: drill down/up, legend toggle, zoom, fullscreen; drill beyond the rows asks a follow-up</t>
+        </is>
+      </c>
+      <c r="C69" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D69" s="14" t="inlineStr">
+        <is>
+          <t>charts.tsx (onDrill wired in Analysis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>Learning, building, agents, graphs and consolidation (Sep 24–25)</t>
+        </is>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>Relationship graph: pan/zoom/drag, focus, source → table → column drill, search, force/hierarchy layout</t>
+        </is>
+      </c>
+      <c r="C70" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D70" s="14" t="inlineStr">
+        <is>
+          <t>GraphCanvas.tsx, RelationshipExplorer.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="14" t="inlineStr">
+        <is>
+          <t>Learning, building, agents, graphs and consolidation (Sep 24–25)</t>
+        </is>
+      </c>
+      <c r="B71" s="14" t="inlineStr">
+        <is>
+          <t>Consolidation: five nav areas, role defaults + "Show advanced", Agents &amp; tools merged, Learning holds all feedback loops, Home opens Analysis, missing safety buttons, one "Save as…" menu</t>
+        </is>
+      </c>
+      <c r="C71" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D71" s="14" t="inlineStr">
+        <is>
+          <t>docs/UX_CONSOLIDATION.md; /tools and /evaluations redirect</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="14" t="inlineStr">
+        <is>
+          <t>Learning, building, agents, graphs and consolidation (Sep 24–25)</t>
+        </is>
+      </c>
+      <c r="B72" s="14" t="inlineStr">
+        <is>
+          <t>Admin → Screens: hide pages or single tabs per project (e.g. for demos); presentation only, audited</t>
+        </is>
+      </c>
+      <c r="C72" s="15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D72" s="14" t="inlineStr">
+        <is>
+          <t>screen_visibility.py, GET/PUT /ui/screens, ScreenVisibilityPanel.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="14" t="inlineStr">
+        <is>
+          <t>Learning, building, agents, graphs and consolidation (Sep 24–25)</t>
+        </is>
+      </c>
+      <c r="B73" s="14" t="inlineStr">
+        <is>
+          <t>Jobs → Retry for tuning / composition / prompt-optimisation jobs</t>
+        </is>
+      </c>
+      <c r="C73" s="15" t="inlineStr">
+        <is>
+          <t>✅ Fixed</t>
+        </is>
+      </c>
+      <c r="D73" s="14" t="inlineStr">
+        <is>
+          <t>Returns where to re-run instead of starting an agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="14" t="inlineStr">
+        <is>
           <t>Still open</t>
         </is>
       </c>
-      <c r="B63" s="14" t="inlineStr">
+      <c r="B74" s="14" t="inlineStr">
+        <is>
+          <t>Rotate the Gemini and OpenRouter API keys shared in chat</t>
+        </is>
+      </c>
+      <c r="C74" s="16" t="inlineStr">
+        <is>
+          <t>🔴 User action</t>
+        </is>
+      </c>
+      <c r="D74" s="14" t="inlineStr">
+        <is>
+          <t>Keys are only in the gitignored .env</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="14" t="inlineStr">
+        <is>
+          <t>Still open</t>
+        </is>
+      </c>
+      <c r="B75" s="14" t="inlineStr">
+        <is>
+          <t>Change the seeded admin's temporary password</t>
+        </is>
+      </c>
+      <c r="C75" s="16" t="inlineStr">
+        <is>
+          <t>🔴 User action</t>
+        </is>
+      </c>
+      <c r="D75" s="14" t="inlineStr">
+        <is>
+          <t>The forced "change temporary password" dialog still appears</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="14" t="inlineStr">
+        <is>
+          <t>Still open</t>
+        </is>
+      </c>
+      <c r="B76" s="14" t="inlineStr">
+        <is>
+          <t>Commit this work</t>
+        </is>
+      </c>
+      <c r="C76" s="16" t="inlineStr">
+        <is>
+          <t>🔴 User action</t>
+        </is>
+      </c>
+      <c r="D76" s="14" t="inlineStr">
+        <is>
+          <t>Nothing has been committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="14" t="inlineStr">
+        <is>
+          <t>Still open</t>
+        </is>
+      </c>
+      <c r="B77" s="14" t="inlineStr">
+        <is>
+          <t>MCP streamable HTTP (GET/SSE)</t>
+        </is>
+      </c>
+      <c r="C77" s="17" t="inlineStr">
+        <is>
+          <t>🟡 By choice</t>
+        </is>
+      </c>
+      <c r="D77" s="14" t="inlineStr">
+        <is>
+          <t>POST JSON-RPC covers current clients</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="14" t="inlineStr">
+        <is>
+          <t>Still open</t>
+        </is>
+      </c>
+      <c r="B78" s="14" t="inlineStr">
+        <is>
+          <t>AgentVersion.input_schema / config at run time</t>
+        </is>
+      </c>
+      <c r="C78" s="17" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="D78" s="14" t="inlineStr">
+        <is>
+          <t>Stored, not yet used</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="14" t="inlineStr">
+        <is>
+          <t>Still open</t>
+        </is>
+      </c>
+      <c r="B79" s="14" t="inlineStr">
+        <is>
+          <t>Timed-out built-in tool threads</t>
+        </is>
+      </c>
+      <c r="C79" s="17" t="inlineStr">
+        <is>
+          <t>🟡 By design</t>
+        </is>
+      </c>
+      <c r="D79" s="14" t="inlineStr">
+        <is>
+          <t>Interrupted at the database; the thread can't be killed</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="14" t="inlineStr">
+        <is>
+          <t>Still open</t>
+        </is>
+      </c>
+      <c r="B80" s="14" t="inlineStr">
         <is>
           <t>Items carried from August (§2): PingFederate SSO, pen test, demo video, connector certification beyond SQL Server</t>
         </is>
       </c>
-      <c r="C63" s="16" t="inlineStr">
+      <c r="C80" s="16" t="inlineStr">
         <is>
           <t>🔴 Unchanged</t>
         </is>
       </c>
-      <c r="D63" s="14" t="inlineStr">
+      <c r="D80" s="14" t="inlineStr">
         <is>
           <t>Outside this review's scope</t>
         </is>

</xml_diff>